<commit_message>
LGSRC 2026/6/8 更新 5
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{875AFEF2-0FEC-4091-94B2-3631A3638364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744A454F-8BAE-4E7E-9F38-FCFE435EA341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
   <si>
     <t>鲁大师</t>
   </si>
@@ -163,6 +163,10 @@
   </si>
   <si>
     <t>酷我音乐</t>
+  </si>
+  <si>
+    <t>DeepL (翻译器)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -487,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A38"/>
+  <dimension ref="A1:A39"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.640625" customWidth="1"/>
@@ -510,182 +514,187 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>3</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
         <v>10</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A38">
-    <sortCondition ref="A38"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A39">
+    <sortCondition ref="A39"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/13 更新 1
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{744A454F-8BAE-4E7E-9F38-FCFE435EA341}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C894DAA-B51B-4365-9560-EC887803772C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
   <si>
     <t>鲁大师</t>
   </si>
@@ -167,6 +167,9 @@
   <si>
     <t>DeepL (翻译器)</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>石墨文档</t>
   </si>
 </sst>
 </file>
@@ -491,7 +494,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A39"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.640625" customWidth="1"/>
@@ -664,37 +667,42 @@
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>10</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A39">
-    <sortCondition ref="A39"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A40">
+    <sortCondition ref="A40"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/13 更新 5
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C894DAA-B51B-4365-9560-EC887803772C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E4F7666-8BFC-4D94-B120-51236234B58A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
   <si>
     <t>鲁大师</t>
   </si>
@@ -170,6 +170,9 @@
   </si>
   <si>
     <t>石墨文档</t>
+  </si>
+  <si>
+    <t>有道云笔记</t>
   </si>
 </sst>
 </file>
@@ -494,7 +497,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.640625" customWidth="1"/>
@@ -700,9 +703,14 @@
         <v>10</v>
       </c>
     </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A40">
-    <sortCondition ref="A40"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A41">
+    <sortCondition ref="A41"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/14 更新 1
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E4F7666-8BFC-4D94-B120-51236234B58A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95402620-F1D4-43E0-AAE7-21282ECFC1B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
   <si>
     <t>鲁大师</t>
   </si>
@@ -173,6 +173,10 @@
   </si>
   <si>
     <t>有道云笔记</t>
+  </si>
+  <si>
+    <t>Xmind (思维导图)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -497,7 +501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A41"/>
+  <dimension ref="A1:A42"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.640625" customWidth="1"/>
@@ -600,117 +604,122 @@
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A41">
-    <sortCondition ref="A41"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A42">
+    <sortCondition ref="A42"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/14 更新 2
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95402620-F1D4-43E0-AAE7-21282ECFC1B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1645BD88-4CCC-4D2F-8F12-4A082032BA29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>鲁大师</t>
   </si>
@@ -176,6 +176,18 @@
   </si>
   <si>
     <t>Xmind (思维导图)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>VPN 工具 (不限开发商)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>网易云音乐</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TeamViewer (远程控制软件)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -501,7 +513,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A42"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.640625" customWidth="1"/>
@@ -589,137 +601,152 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>3</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>8</v>
+        <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>2</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>1</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>37</v>
+        <v>17</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>0</v>
+        <v>37</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>22</v>
+        <v>34</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A42">
-    <sortCondition ref="A42"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A45">
+    <sortCondition ref="A45"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/14 更新 3
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1645BD88-4CCC-4D2F-8F12-4A082032BA29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FB26B48-B9CD-478D-B42F-9BF9B5961A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>鲁大师</t>
   </si>
@@ -188,6 +188,10 @@
   </si>
   <si>
     <t>TeamViewer (远程控制软件)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>剪映 (字节跳动)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -513,7 +517,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="26.640625" customWidth="1"/>
@@ -666,87 +670,92 @@
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>43</v>
+        <v>16</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A45">
-    <sortCondition ref="A45"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A46">
+    <sortCondition ref="A46"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/14 更新 5
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FB26B48-B9CD-478D-B42F-9BF9B5961A21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F3CF2B9-E45C-412A-8F22-A07823E4EB38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t>鲁大师</t>
   </si>
@@ -193,6 +193,12 @@
   <si>
     <t>剪映 (字节跳动)</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>百度网盘</t>
+  </si>
+  <si>
+    <t>阿里云盘</t>
   </si>
 </sst>
 </file>
@@ -517,245 +523,255 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A46"/>
-  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:A48"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.640625" customWidth="1"/>
+    <col min="1" max="1" width="30.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A46">
-    <sortCondition ref="A46"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A48">
+    <sortCondition ref="A48"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/15 更新 5
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66746BC9-CA48-4877-B41A-82B7D30A1C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -532,257 +532,257 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A50"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.77734375" customWidth="1"/>
+    <col min="1" max="1" width="30.78515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>40</v>
       </c>

</xml_diff>

<commit_message>
LGSRC 2026/6/16 更新 3
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66746BC9-CA48-4877-B41A-82B7D30A1C80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A673C9-36F1-4218-B748-11EDABB21AEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>鲁大师</t>
   </si>
@@ -206,6 +206,10 @@
   </si>
   <si>
     <t>迅游网游加速器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>WeGame (游戏平台)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -531,265 +535,270 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A50"/>
-  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:A51"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.78515625" customWidth="1"/>
+    <col min="1" max="1" width="30.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A50">
-    <sortCondition ref="A50"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A51">
+    <sortCondition ref="A51"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/16 更新 5
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A673C9-36F1-4218-B748-11EDABB21AEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73528322-BF05-4CEF-BFE9-B352AC7AE54D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
   <si>
     <t>鲁大师</t>
   </si>
@@ -210,6 +210,10 @@
   </si>
   <si>
     <t>WeGame (游戏平台)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BitComet (比特彗星)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -535,7 +539,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A51"/>
+  <dimension ref="A1:A52"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.77734375" customWidth="1"/>
@@ -553,252 +557,257 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>3</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>42</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>41</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>45</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>39</v>
+        <v>4</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A51">
-    <sortCondition ref="A51"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A52">
+    <sortCondition ref="A52"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/17 更新 1
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73528322-BF05-4CEF-BFE9-B352AC7AE54D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A7272EA-27C6-46C3-A784-104E4C429748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>鲁大师</t>
   </si>
@@ -215,6 +215,12 @@
   <si>
     <t>BitComet (比特彗星)</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>驱动总裁</t>
+  </si>
+  <si>
+    <t>驱动精灵</t>
   </si>
 </sst>
 </file>
@@ -539,7 +545,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A52"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.77734375" customWidth="1"/>
@@ -752,62 +758,72 @@
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>7</v>
+        <v>52</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>48</v>
+        <v>25</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>43</v>
+        <v>16</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>29</v>
+        <v>48</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A52">
-    <sortCondition ref="A52"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A54">
+    <sortCondition ref="A54"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/17 更新 2
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A7272EA-27C6-46C3-A784-104E4C429748}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334349A1-FB10-44DD-A539-0138C62C612D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
   <si>
     <t>鲁大师</t>
   </si>
@@ -221,6 +221,10 @@
   </si>
   <si>
     <t>驱动精灵</t>
+  </si>
+  <si>
+    <t>AnyDesk (远程桌面软件)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -545,7 +549,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A54"/>
+  <dimension ref="A1:A55"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.77734375" customWidth="1"/>
@@ -563,267 +567,272 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>3</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>42</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>41</v>
+        <v>5</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>45</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>53</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A54">
-    <sortCondition ref="A54"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A55">
+    <sortCondition ref="A55"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/17 更新 3
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{334349A1-FB10-44DD-A539-0138C62C612D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C740758D-9425-4DFF-AE13-127A1DA05A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
   <si>
     <t>鲁大师</t>
   </si>
@@ -225,6 +225,9 @@
   <si>
     <t>AnyDesk (远程桌面软件)</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2345 浏览器</t>
   </si>
 </sst>
 </file>
@@ -549,7 +552,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A55"/>
+  <dimension ref="A1:A56"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.77734375" customWidth="1"/>
@@ -557,282 +560,287 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>54</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>14</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>3</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>41</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>30</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>45</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>0</v>
+        <v>34</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>53</v>
+        <v>4</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A55">
-    <sortCondition ref="A55"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A56">
+    <sortCondition ref="A56"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/18 更新 1
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C740758D-9425-4DFF-AE13-127A1DA05A90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFCF24B6-DB4D-43AC-BC07-4B3539FDF367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
   <si>
     <t>鲁大师</t>
   </si>
@@ -228,6 +228,10 @@
   </si>
   <si>
     <t>2345 浏览器</t>
+  </si>
+  <si>
+    <t>夸克网盘</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -552,7 +556,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A56"/>
+  <dimension ref="A1:A57"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.77734375" customWidth="1"/>
@@ -760,87 +764,92 @@
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>0</v>
+        <v>56</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>53</v>
+        <v>4</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A56">
-    <sortCondition ref="A56"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A57">
+    <sortCondition ref="A57"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/19 更新 1
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFCF24B6-DB4D-43AC-BC07-4B3539FDF367}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4DA0ECF-AAB9-40BA-B246-6F9E4A5B434C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
   <si>
     <t>鲁大师</t>
   </si>
@@ -231,6 +231,49 @@
   </si>
   <si>
     <t>夸克网盘</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>比特浏览器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>WinRAR</t>
+  </si>
+  <si>
+    <t>悟空浏览器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>小红书</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>BlueStacks (安卓模拟器)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>WhatsApp (即时通讯软件)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Xchat (即时通讯软件)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>腾讯文档</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>搜狗浏览器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MT5 (金融交易平台)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Canva 可画 (设计平台)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -556,7 +599,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A57"/>
+  <dimension ref="A1:A68"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.77734375" customWidth="1"/>
@@ -845,6 +888,61 @@
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>40</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
LGSRC 2026/6/19 更新 2
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4DA0ECF-AAB9-40BA-B246-6F9E4A5B434C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEA95E3F-19E3-4340-BFF4-7DE5936A5DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -632,322 +632,322 @@
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>28</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>44</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>3</v>
+        <v>27</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>8</v>
+        <v>58</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>46</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>6</v>
+        <v>63</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>2</v>
+        <v>21</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>17</v>
+        <v>6</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>4</v>
+        <v>17</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>52</v>
+        <v>37</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>7</v>
+        <v>56</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>25</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>29</v>
+        <v>52</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>49</v>
+        <v>39</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>23</v>
+        <v>65</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>63</v>
+        <v>29</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>66</v>
+        <v>10</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>67</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A57">
-    <sortCondition ref="A57"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A68">
+    <sortCondition ref="A1:A68"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/19 更新 3
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEA95E3F-19E3-4340-BFF4-7DE5936A5DDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A53FDEE8-ADFC-408D-BC16-55F89125A39B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
   <si>
     <t>鲁大师</t>
   </si>
@@ -274,6 +274,10 @@
   </si>
   <si>
     <t>Canva 可画 (设计平台)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>KOOK (语音沟通工具)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -599,7 +603,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A68"/>
+  <dimension ref="A1:A69"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.77734375" customWidth="1"/>
@@ -687,267 +691,272 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>14</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>66</v>
+        <v>11</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>3</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>42</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>62</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>5</v>
+        <v>58</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>63</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>41</v>
+        <v>63</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>8</v>
+        <v>21</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>6</v>
+        <v>46</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>57</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>30</v>
+        <v>57</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>45</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>0</v>
+        <v>56</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>53</v>
+        <v>4</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>65</v>
+        <v>39</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>7</v>
+        <v>65</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>64</v>
+        <v>25</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>16</v>
+        <v>64</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>29</v>
+        <v>60</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>49</v>
+        <v>29</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>23</v>
+        <v>49</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A68">
-    <sortCondition ref="A1:A68"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A69">
+    <sortCondition ref="A69"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/19 更新 5
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A53FDEE8-ADFC-408D-BC16-55F89125A39B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4027E630-91EC-4C55-8AFD-D4767866C231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
   <si>
     <t>鲁大师</t>
   </si>
@@ -279,6 +279,28 @@
   <si>
     <t>KOOK (语音沟通工具)</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UC 浏览器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>网易 MuMu 模拟器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>雷电模拟器</t>
+  </si>
+  <si>
+    <t>Hubstudio (浏览器)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SafeW (即时通讯软件)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>金山词霸</t>
   </si>
 </sst>
 </file>
@@ -603,7 +625,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A69"/>
+  <dimension ref="A1:A75"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.77734375" customWidth="1"/>
@@ -691,272 +713,302 @@
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>14</v>
+        <v>68</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>66</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>44</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>3</v>
+        <v>44</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>50</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>5</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>41</v>
+        <v>58</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>47</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>21</v>
+        <v>63</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>8</v>
+        <v>41</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>57</v>
+        <v>8</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>30</v>
+        <v>46</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>2</v>
+        <v>57</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>1</v>
+        <v>30</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>45</v>
+        <v>20</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>17</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>36</v>
+        <v>1</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>34</v>
+        <v>74</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>56</v>
+        <v>17</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>22</v>
+        <v>37</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>4</v>
+        <v>34</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>39</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>65</v>
+        <v>22</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>25</v>
+        <v>53</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>16</v>
+        <v>39</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>43</v>
+        <v>7</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>59</v>
+        <v>25</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>49</v>
+        <v>70</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>10</v>
+        <v>43</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>40</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A69">
-    <sortCondition ref="A69"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A75">
+    <sortCondition ref="A75"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/19 更新 8
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36C6BFE3-E9E8-414F-AE98-8BD18AEDA3A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFD92E3C-EF0A-4891-9A49-C14B754F959E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
   <si>
     <t>鲁大师</t>
   </si>
@@ -101,10 +101,6 @@
     <t>360 安全浏览器</t>
   </si>
   <si>
-    <t>豆包桌面版</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>爱翻译</t>
   </si>
   <si>
@@ -330,6 +326,21 @@
   <si>
     <t>网易 UU 远程</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>千问 AI</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>豆包 AI</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Signal (即时通讯软件)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>紫鸟浏览器</t>
   </si>
 </sst>
 </file>
@@ -654,7 +665,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A83"/>
+  <dimension ref="A1:A86"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.77734375" customWidth="1"/>
@@ -662,7 +673,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -677,47 +688,47 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
@@ -737,22 +748,22 @@
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
@@ -767,7 +778,7 @@
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
@@ -777,287 +788,287 @@
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>27</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>3</v>
+        <v>34</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>69</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>42</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>62</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>5</v>
+        <v>57</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>63</v>
+        <v>5</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>41</v>
+        <v>62</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>76</v>
+        <v>40</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>47</v>
+        <v>75</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>46</v>
+        <v>8</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>57</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>30</v>
+        <v>56</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>2</v>
+        <v>83</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>45</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>77</v>
+        <v>44</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>17</v>
+        <v>73</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>56</v>
+        <v>33</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>22</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>81</v>
+        <v>21</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>53</v>
+        <v>4</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>52</v>
+        <v>82</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>65</v>
+        <v>51</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>25</v>
+        <v>64</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>64</v>
+        <v>7</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>59</v>
+        <v>81</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>80</v>
+        <v>42</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>29</v>
+        <v>79</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>49</v>
+        <v>59</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>79</v>
+        <v>28</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>23</v>
+        <v>48</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
@@ -1067,17 +1078,32 @@
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>40</v>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A83">
-    <sortCondition ref="A1:A83"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A86">
+    <sortCondition ref="A86"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/19 更新 9
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFD92E3C-EF0A-4891-9A49-C14B754F959E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB648F9-5780-42A4-8BBC-0ABC86D8F3FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="89">
   <si>
     <t>鲁大师</t>
   </si>
@@ -341,6 +341,17 @@
   </si>
   <si>
     <t>紫鸟浏览器</t>
+  </si>
+  <si>
+    <t>创客贴 (设计平台)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>稿定设计</t>
+  </si>
+  <si>
+    <t>SketchUp (3D 设计软件)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -665,7 +676,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A86"/>
+  <dimension ref="A1:A89"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.77734375" customWidth="1"/>
@@ -803,307 +814,322 @@
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>26</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>3</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>68</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>5</v>
+        <v>57</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>62</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>75</v>
+        <v>40</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>29</v>
+        <v>56</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>2</v>
+        <v>29</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>1</v>
+        <v>83</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>44</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>73</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>17</v>
+        <v>44</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>36</v>
+        <v>73</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>55</v>
+        <v>35</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>70</v>
+        <v>36</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>0</v>
+        <v>33</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>21</v>
+        <v>55</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>80</v>
+        <v>70</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>82</v>
+        <v>21</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>52</v>
+        <v>80</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>51</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>38</v>
+        <v>82</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>64</v>
+        <v>52</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>7</v>
+        <v>51</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>69</v>
+        <v>24</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>81</v>
+        <v>16</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>42</v>
+        <v>69</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>28</v>
+        <v>58</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>77</v>
+        <v>48</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>10</v>
+        <v>78</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A86">
-    <sortCondition ref="A86"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A89">
+    <sortCondition ref="A89"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/19 更新 10
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BB648F9-5780-42A4-8BBC-0ABC86D8F3FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB885D94-DE05-43DF-9A89-DD67B82F4AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
   <si>
     <t>鲁大师</t>
   </si>
@@ -351,6 +351,10 @@
   </si>
   <si>
     <t>SketchUp (3D 设计软件)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>元宝 AI</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -676,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A89"/>
+  <dimension ref="A1:A90"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30.77734375" customWidth="1"/>
@@ -1124,12 +1128,17 @@
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A89">
-    <sortCondition ref="A89"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A90">
+    <sortCondition ref="A90"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/19 更新 11
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB885D94-DE05-43DF-9A89-DD67B82F4AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{476CE618-4898-4B4E-988A-8FF605364B59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
   <si>
     <t>鲁大师</t>
   </si>
@@ -355,6 +355,17 @@
   </si>
   <si>
     <t>元宝 AI</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Letstalk (加密通讯软件)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>驱动天空</t>
+  </si>
+  <si>
+    <t>Radmin (远程桌面软件)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -680,465 +691,480 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A90"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A93"/>
+  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.77734375" customWidth="1"/>
+    <col min="1" max="1" width="30.78515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A46" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A49" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A50" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A51" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A52" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A53" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A54" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A90">
-    <sortCondition ref="A90"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A93">
+    <sortCondition ref="A93"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/19 更新 12
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{476CE618-4898-4B4E-988A-8FF605364B59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF169EFF-2605-4819-989E-9BA52646CB07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
   <si>
     <t>鲁大师</t>
   </si>
@@ -366,6 +366,10 @@
   </si>
   <si>
     <t>Radmin (远程桌面软件)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>QQ 音乐</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -691,7 +695,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A93"/>
+  <dimension ref="A1:A94"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.78515625" customWidth="1"/>
@@ -824,347 +828,352 @@
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>26</v>
+        <v>88</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>3</v>
+        <v>34</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>68</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>5</v>
+        <v>57</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>62</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>75</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>86</v>
+        <v>56</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>29</v>
+        <v>86</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>2</v>
+        <v>83</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>87</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>1</v>
+        <v>87</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>44</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>76</v>
+        <v>44</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>17</v>
+        <v>73</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>55</v>
+        <v>33</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>0</v>
+        <v>70</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>21</v>
+        <v>0</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>80</v>
+        <v>21</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>82</v>
+        <v>4</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>52</v>
+        <v>82</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>91</v>
+        <v>52</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>51</v>
+        <v>91</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>64</v>
+        <v>38</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>7</v>
+        <v>64</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>24</v>
+        <v>7</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>63</v>
+        <v>24</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>16</v>
+        <v>63</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>69</v>
+        <v>16</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>47</v>
+        <v>69</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>81</v>
+        <v>47</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>42</v>
+        <v>81</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>59</v>
+        <v>79</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>22</v>
+        <v>78</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>77</v>
+        <v>22</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>10</v>
+        <v>77</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>89</v>
+        <v>39</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A93">
-    <sortCondition ref="A93"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A94">
+    <sortCondition ref="A94"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/20 更新 1
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF169EFF-2605-4819-989E-9BA52646CB07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80D6AF95-A9D8-45E8-96E2-A095CED7823F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
   <si>
     <t>鲁大师</t>
   </si>
@@ -371,6 +371,9 @@
   <si>
     <t>QQ 音乐</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>希沃白板</t>
   </si>
 </sst>
 </file>
@@ -695,7 +698,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A94"/>
+  <dimension ref="A1:A95"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.78515625" customWidth="1"/>
@@ -1118,62 +1121,67 @@
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>79</v>
+        <v>94</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>59</v>
+        <v>79</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>28</v>
+        <v>59</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>48</v>
+        <v>28</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>78</v>
+        <v>48</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>22</v>
+        <v>78</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>77</v>
+        <v>22</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>10</v>
+        <v>77</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>39</v>
+        <v>10</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>89</v>
+        <v>39</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A94">
-    <sortCondition ref="A94"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A95">
+    <sortCondition ref="A95"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/20 更新 2
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80D6AF95-A9D8-45E8-96E2-A095CED7823F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F627D4-07F3-42C3-B171-7E1F086B8F0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="97">
   <si>
     <t>鲁大师</t>
   </si>
@@ -374,6 +374,14 @@
   </si>
   <si>
     <t>希沃白板</t>
+  </si>
+  <si>
+    <t>福昕 PDF 阅读器</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>360 压缩</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -698,7 +706,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A95"/>
+  <dimension ref="A1:A97"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.78515625" customWidth="1"/>
@@ -721,467 +729,477 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>96</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>27</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>71</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>90</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>90</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>65</v>
+        <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>93</v>
+        <v>30</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>72</v>
+        <v>92</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>84</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>26</v>
+        <v>88</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>3</v>
+        <v>34</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>68</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>41</v>
+        <v>68</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>5</v>
+        <v>57</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>62</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>75</v>
+        <v>40</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>46</v>
+        <v>75</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>86</v>
+        <v>56</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>29</v>
+        <v>86</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>2</v>
+        <v>83</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>87</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>1</v>
+        <v>95</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>44</v>
+        <v>87</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>76</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>73</v>
+        <v>44</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>17</v>
+        <v>76</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>70</v>
+        <v>33</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>0</v>
+        <v>55</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>52</v>
+        <v>4</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>38</v>
+        <v>91</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>24</v>
+        <v>64</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>63</v>
+        <v>7</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>94</v>
+        <v>42</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>59</v>
+        <v>94</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>28</v>
+        <v>79</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>89</v>
+        <v>10</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A95">
-    <sortCondition ref="A95"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A97">
+    <sortCondition ref="A97"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/22 更新 3
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37F627D4-07F3-42C3-B171-7E1F086B8F0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231287AC-3E04-4D59-BD72-0269A4F754BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
   <si>
     <t>鲁大师</t>
   </si>
@@ -381,6 +381,14 @@
   </si>
   <si>
     <t>360 压缩</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>虎牙直播</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>按键精灵</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -706,7 +714,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A97"/>
+  <dimension ref="A1:A99"/>
   <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="30.78515625" customWidth="1"/>
@@ -949,257 +957,267 @@
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>45</v>
+        <v>98</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>6</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>56</v>
+        <v>6</v>
       </c>
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>86</v>
+        <v>56</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>29</v>
+        <v>86</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>2</v>
+        <v>83</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>95</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>1</v>
+        <v>87</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>44</v>
+        <v>97</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>76</v>
+        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>73</v>
+        <v>44</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>17</v>
+        <v>76</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>55</v>
+        <v>36</v>
       </c>
     </row>
     <row r="66" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>70</v>
+        <v>33</v>
       </c>
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>0</v>
+        <v>55</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>21</v>
+        <v>70</v>
       </c>
     </row>
     <row r="69" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>80</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
     </row>
     <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>52</v>
+        <v>4</v>
       </c>
     </row>
     <row r="73" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="75" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>38</v>
+        <v>91</v>
       </c>
     </row>
     <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>24</v>
+        <v>64</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>63</v>
+        <v>7</v>
       </c>
     </row>
     <row r="80" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>47</v>
+        <v>16</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>58</v>
+        <v>81</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
-        <v>94</v>
+        <v>42</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
-        <v>79</v>
+        <v>58</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
-        <v>59</v>
+        <v>94</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
-        <v>28</v>
+        <v>79</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
-        <v>48</v>
+        <v>59</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
-        <v>78</v>
+        <v>28</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
-        <v>89</v>
+        <v>10</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A97">
-    <sortCondition ref="A97"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A99">
+    <sortCondition ref="A99"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/6/26 更新 5
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{231287AC-3E04-4D59-BD72-0269A4F754BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE889086-B3F2-4DDE-9828-CF6867F363C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="101">
   <si>
     <t>鲁大师</t>
   </si>
@@ -390,6 +390,12 @@
   <si>
     <t>按键精灵</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>7-Zip</t>
+  </si>
+  <si>
+    <t>Bandizip</t>
   </si>
 </sst>
 </file>
@@ -714,510 +720,520 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A99"/>
-  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:A101"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.78515625" customWidth="1"/>
+    <col min="1" max="1" width="30.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A86" t="s">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A87" t="s">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A89" t="s">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A90" t="s">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A91" t="s">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A92" t="s">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A94" t="s">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A95" t="s">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A96" t="s">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A97" t="s">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A99">
-    <sortCondition ref="A99"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A101">
+    <sortCondition ref="A101"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/8/15 更新 5
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{756E19F8-F6A7-4F2E-9141-E2B25460B981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{052EBCA3-4093-4241-9A12-EF56BE269938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
   <si>
     <t>鲁大师</t>
   </si>
@@ -399,6 +399,10 @@
   </si>
   <si>
     <t>讯飞输入法</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>豆包输入法</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -724,525 +728,530 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A102"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A103"/>
+  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.77734375" customWidth="1"/>
+    <col min="1" max="1" width="30.78515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A102">
-    <sortCondition ref="A102"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A103">
+    <sortCondition ref="A103"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/8/19 更新 2
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{052EBCA3-4093-4241-9A12-EF56BE269938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5032155F-E878-4903-A747-D2DA370D6992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
   <si>
     <t>鲁大师</t>
   </si>
@@ -403,6 +403,14 @@
   </si>
   <si>
     <t>豆包输入法</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>金山毒霸</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>金山打字通</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -728,530 +736,540 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A103"/>
-  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:A105"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.78515625" customWidth="1"/>
+    <col min="1" max="1" width="30.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A86" t="s">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A87" t="s">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A89" t="s">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A90" t="s">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A91" t="s">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A92" t="s">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A94" t="s">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A95" t="s">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A96" t="s">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A97" t="s">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A100" t="s">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A101" t="s">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A102" t="s">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A103" t="s">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A103">
-    <sortCondition ref="A103"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A105">
+    <sortCondition ref="A105"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/8/24 更新 2
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5032155F-E878-4903-A747-D2DA370D6992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{389976B4-99A8-44C0-9B32-9E2D7732E3CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
   <si>
     <t>鲁大师</t>
   </si>
@@ -411,6 +411,13 @@
   </si>
   <si>
     <t>金山打字通</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>必剪</t>
+  </si>
+  <si>
+    <t>卡巴斯基</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -736,540 +743,550 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A105"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A107"/>
+  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.77734375" customWidth="1"/>
+    <col min="1" max="1" width="30.78515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A55" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A56" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A57" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A58" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A59" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A60" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A61" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A62" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A64" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A65" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A66" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A67" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A70" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A71" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A72" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A74" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A77" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A77" t="s">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A85" t="s">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A87" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A86" t="s">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A88" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A87" t="s">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A89" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A88" t="s">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A90" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A89" t="s">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A90" t="s">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A105">
-    <sortCondition ref="A105"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A107">
+    <sortCondition ref="A107"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/8/27 更新 3
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{389976B4-99A8-44C0-9B32-9E2D7732E3CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774D9A7B-ABAA-446B-AD7B-591FBA6968AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
   <si>
     <t>鲁大师</t>
   </si>
@@ -418,6 +418,10 @@
   </si>
   <si>
     <t>卡巴斯基</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Brave (浏览器)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -743,550 +747,555 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A107"/>
-  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:A108"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="30.78515625" customWidth="1"/>
+    <col min="1" max="1" width="30.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A48" t="s">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" t="s">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A50" t="s">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A51" t="s">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A52" t="s">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A53" t="s">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A54" t="s">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A55" t="s">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A56" t="s">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A57" t="s">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A58" t="s">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A59" t="s">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A60" t="s">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A61" t="s">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A62" t="s">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A71" t="s">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A86" t="s">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A87" t="s">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A89" t="s">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A90" t="s">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A91" t="s">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A92" t="s">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A93" t="s">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A94" t="s">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A95" t="s">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A96" t="s">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A97" t="s">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A98" t="s">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A99" t="s">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A100" t="s">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A101" t="s">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A102" t="s">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A103" t="s">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A104" t="s">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A105" t="s">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A106" t="s">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A107" t="s">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A107">
-    <sortCondition ref="A107"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A108">
+    <sortCondition ref="A108"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
LGSRC 2026/8/28 更新 1
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{774D9A7B-ABAA-446B-AD7B-591FBA6968AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4925ED7F-4D6D-458F-B7FE-8F2547A31A20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="软件列表" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>

</xml_diff>

<commit_message>
LGSRC 2026/9/5 更新 2
签发：Ling Gao (LGSRC)
</commit_message>
<xml_diff>
--- a/Documents/List.xlsx
+++ b/Documents/List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hnist\Desktop\LGSRC\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4925ED7F-4D6D-458F-B7FE-8F2547A31A20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98550B2D-8B55-4D0F-8B11-B1A2BCA26654}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="19954" windowHeight="12652" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="软件列表" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
   <si>
     <t>鲁大师</t>
   </si>
@@ -422,6 +422,10 @@
   </si>
   <si>
     <t>Brave (浏览器)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>同花顺 (金融软件)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -747,555 +751,560 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A108"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:A109"/>
+  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.77734375" customWidth="1"/>
+    <col min="1" max="1" width="30.78515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A91" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" t="s">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A92" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A92" t="s">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A93" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A93" t="s">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A94" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A94" t="s">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A95" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A95" t="s">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A96" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A96" t="s">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A97" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A97" t="s">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A98" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A98" t="s">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A99" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A99" t="s">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A100" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A100" t="s">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A101" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A101" t="s">
+    <row r="102" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A102" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
+    <row r="103" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A103" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A103" t="s">
+    <row r="104" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A104" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A104" t="s">
+    <row r="105" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A105" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A105" t="s">
+    <row r="106" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A106" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A106" t="s">
+    <row r="107" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A107" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A107" t="s">
+    <row r="108" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A108" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A108" t="s">
+    <row r="109" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A109" t="s">
         <v>85</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A108">
-    <sortCondition ref="A108"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A109">
+    <sortCondition ref="A109"/>
   </sortState>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>